<commit_message>
docs: add pages template and api bug reports
</commit_message>
<xml_diff>
--- a/documents/СПО_Goblincore_Список_API.xlsx
+++ b/documents/СПО_Goblincore_Список_API.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kseni\Downloads\University\Software_development_5_sem\Goblincore\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC568B55-B493-49DD-BAA1-7F4AA023BBF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E0A9669-BCC2-46B8-8741-A638CB76400D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1590AC1E-9868-44FB-9EAB-05B7C1F3B120}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="103">
   <si>
     <t>№</t>
   </si>
@@ -298,6 +298,116 @@
   </si>
   <si>
     <t>q, page, limit</t>
+  </si>
+  <si>
+    <t>400 - невалидный email или пустой username
+409 - email уже зарегистрирован
+422 - пропущены обязательные поля
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>400 - неверный grant_type
+401 - неверный username или password_hash
+422 - пропущены обязательные поля
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>400 - неверный grant_type
+401 - refresh_token недействителен или истёк
+422 - пропущено поле refresh_token
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>401 - нет токена авторизации
+403 - попытка получить чужой профиль
+404 - пользователь не найден
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>400 - невалидные данные
+401 - нет токена авторизации
+403 - попытка изменить чужой профиль
+404 - пользователь не найден
+409 - новый email уже занят
+422 - пропущены обязательные поля
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>401 - нет токена авторизации
+403 - попытка удалить чужой аккаунт
+404 - пользователь не найден
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>400 - неверный transaction_type (не income и не expense)
+401 - нет токена авторизации
+403 - попытка получить чужие транзакции
+404 - пользователь не найден
+422 - неверный формат start_date или end_date
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>400 - неверный transaction_type
+401 - нет токена авторизации
+403 - попытка создать транзакцию для другого пользователя
+404 - place_id или category_id не найдены
+422 - пропущены обязательные поля, неверный формат даты или суммы
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>400 - неверный transaction_type
+401 - нет токена авторизации
+403 - попытка изменить чужую транзакцию
+404 - транзакция, place_id или category_id не найдены
+422 - неверный формат полей
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>400 - неверный transaction_type
+401 - нет токена авторизации
+403 - попытка удалить чужую транзакцию
+404 - транзакция не найдена
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>400 - неверный transaction_type
+401 - нет токена авторизации
+403 - попытка получить чужие категории
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>401 - нет токена авторизации
+403 - попытка создать категорию для другого пользователя
+422 - пропущены обязательные поля
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>401 - нет токена авторизации
+403 - попытка создать категорию для другого пользователя
+422 - пропущены обязательные поля или неверный формат limit
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>401 - нет токена авторизации
+403 - попытка изменить чужую категорию
+404 - категория не найдена
+422 - неверный формат полей
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>401 - нет токена авторизации
+403 - попытка изменить чужую категорию
+404 - категория не найдена
+422 - неверный формат полей или limit
+500 - ошибка сервера</t>
+  </si>
+  <si>
+    <t>400 - неверный transaction_type
+401 - нет токена авторизации
+403 - попытка удалить чужую категорию
+404 - категория не найдена
+409 - к категории привязаны транзакции
+500 - ошибка сервера</t>
   </si>
 </sst>
 </file>
@@ -357,12 +467,6 @@
   </cellStyles>
   <dxfs count="10">
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -386,6 +490,12 @@
     <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -400,17 +510,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{964CA5F2-F798-4D02-AE13-E06D74519EE6}" name="Таблица2" displayName="Таблица2" ref="F3:M23" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{964CA5F2-F798-4D02-AE13-E06D74519EE6}" name="Таблица2" displayName="Таблица2" ref="F3:M23" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="F3:M23" xr:uid="{964CA5F2-F798-4D02-AE13-E06D74519EE6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{E9D18DDE-F78C-407D-8EAE-384A5F8E0C51}" name="№" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{A5CD4C8C-3FF0-4897-8959-333DE653E098}" name="Метод" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{EB259A20-CA36-4BC8-A247-9F633143A97E}" name="Путь" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{C233754B-9F4A-4E67-A865-7F1A8B8AA9FC}" name="Тело запроса" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{E51DF80B-EC9A-406E-B4A5-138DB26E42D0}" name="Тело ответа" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{CD926DC4-1B42-431F-8E09-E6C0C93CCF6C}" name="Параметры запроса" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{6C701872-E974-4374-B3F4-231696F8F524}" name="Ошибки" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{02DAF013-6E01-4142-A5DA-D5097E75885C}" name="Назначение" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{E9D18DDE-F78C-407D-8EAE-384A5F8E0C51}" name="№" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{A5CD4C8C-3FF0-4897-8959-333DE653E098}" name="Метод" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{EB259A20-CA36-4BC8-A247-9F633143A97E}" name="Путь" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{C233754B-9F4A-4E67-A865-7F1A8B8AA9FC}" name="Тело запроса" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{E51DF80B-EC9A-406E-B4A5-138DB26E42D0}" name="Тело ответа" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{CD926DC4-1B42-431F-8E09-E6C0C93CCF6C}" name="Параметры запроса" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{6C701872-E974-4374-B3F4-231696F8F524}" name="Ошибки" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{02DAF013-6E01-4142-A5DA-D5097E75885C}" name="Назначение" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -743,7 +853,7 @@
     <col min="9" max="9" width="21.81640625" customWidth="1"/>
     <col min="10" max="10" width="18.36328125" customWidth="1"/>
     <col min="11" max="11" width="19.6328125" customWidth="1"/>
-    <col min="12" max="12" width="14.1796875" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
     <col min="13" max="13" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -815,10 +925,10 @@
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+      <c r="L4" s="5"/>
       <c r="M4" s="4"/>
     </row>
-    <row r="5" spans="2:13" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:13" ht="101.5" x14ac:dyDescent="0.35">
       <c r="B5" s="2">
         <v>2</v>
       </c>
@@ -847,12 +957,14 @@
         <v>80</v>
       </c>
       <c r="K5" s="5"/>
-      <c r="L5" s="4"/>
+      <c r="L5" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="M5" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="2:13" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:13" ht="116" x14ac:dyDescent="0.35">
       <c r="B6" s="2">
         <v>3</v>
       </c>
@@ -883,12 +995,14 @@
       <c r="K6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="L6" s="4"/>
+      <c r="L6" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="M6" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="2:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:13" ht="116" x14ac:dyDescent="0.35">
       <c r="B7" s="2">
         <v>4</v>
       </c>
@@ -919,7 +1033,9 @@
       <c r="K7" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="L7" s="4"/>
+      <c r="L7" s="5" t="s">
+        <v>89</v>
+      </c>
       <c r="M7" s="5" t="s">
         <v>22</v>
       </c>
@@ -945,10 +1061,10 @@
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
+      <c r="L8" s="5"/>
       <c r="M8" s="4"/>
     </row>
-    <row r="9" spans="2:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:13" ht="101.5" x14ac:dyDescent="0.35">
       <c r="B9" s="2">
         <v>6</v>
       </c>
@@ -975,12 +1091,14 @@
         <v>78</v>
       </c>
       <c r="K9" s="5"/>
-      <c r="L9" s="4"/>
+      <c r="L9" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="M9" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="2:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:13" ht="188.5" x14ac:dyDescent="0.35">
       <c r="B10" s="1"/>
       <c r="F10" s="4">
         <v>5</v>
@@ -998,12 +1116,14 @@
         <v>78</v>
       </c>
       <c r="K10" s="5"/>
-      <c r="L10" s="4"/>
+      <c r="L10" s="5" t="s">
+        <v>91</v>
+      </c>
       <c r="M10" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="2:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:13" ht="101.5" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>35</v>
       </c>
@@ -1022,7 +1142,9 @@
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
-      <c r="L11" s="4"/>
+      <c r="L11" s="5" t="s">
+        <v>92</v>
+      </c>
       <c r="M11" s="5" t="s">
         <v>28</v>
       </c>
@@ -1051,7 +1173,7 @@
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
     </row>
-    <row r="13" spans="2:13" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:13" ht="174" x14ac:dyDescent="0.35">
       <c r="B13" s="2">
         <v>7</v>
       </c>
@@ -1082,12 +1204,14 @@
       <c r="K13" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="L13" s="4"/>
+      <c r="L13" s="5" t="s">
+        <v>93</v>
+      </c>
       <c r="M13" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="2:13" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:13" ht="203" x14ac:dyDescent="0.35">
       <c r="B14" s="2">
         <v>8</v>
       </c>
@@ -1116,12 +1240,14 @@
         <v>82</v>
       </c>
       <c r="K14" s="5"/>
-      <c r="L14" s="4"/>
+      <c r="L14" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="M14" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="2:13" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:13" ht="174" x14ac:dyDescent="0.35">
       <c r="B15" s="2">
         <v>9</v>
       </c>
@@ -1150,12 +1276,14 @@
         <v>82</v>
       </c>
       <c r="K15" s="5"/>
-      <c r="L15" s="4"/>
+      <c r="L15" s="5" t="s">
+        <v>95</v>
+      </c>
       <c r="M15" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="2:13" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:13" ht="130.5" x14ac:dyDescent="0.35">
       <c r="B16" s="1"/>
       <c r="F16" s="4">
         <v>10</v>
@@ -1171,7 +1299,9 @@
       </c>
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
-      <c r="L16" s="4"/>
+      <c r="L16" s="5" t="s">
+        <v>96</v>
+      </c>
       <c r="M16" s="5" t="s">
         <v>59</v>
       </c>
@@ -1194,7 +1324,7 @@
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
     </row>
-    <row r="18" spans="2:13" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:13" ht="101.5" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>0</v>
       </c>
@@ -1223,12 +1353,14 @@
         <v>83</v>
       </c>
       <c r="K18" s="5"/>
-      <c r="L18" s="4"/>
+      <c r="L18" s="5" t="s">
+        <v>97</v>
+      </c>
       <c r="M18" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="2:13" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:13" ht="116" x14ac:dyDescent="0.35">
       <c r="B19" s="2">
         <v>10</v>
       </c>
@@ -1257,12 +1389,14 @@
         <v>84</v>
       </c>
       <c r="K19" s="5"/>
-      <c r="L19" s="4"/>
+      <c r="L19" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="M19" s="5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="2:13" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:13" ht="130.5" x14ac:dyDescent="0.35">
       <c r="B20" s="2">
         <v>11</v>
       </c>
@@ -1291,12 +1425,14 @@
         <v>85</v>
       </c>
       <c r="K20" s="5"/>
-      <c r="L20" s="4"/>
+      <c r="L20" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="M20" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="2:13" ht="58" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:13" ht="130.5" x14ac:dyDescent="0.35">
       <c r="B21" s="2">
         <v>12</v>
       </c>
@@ -1325,12 +1461,14 @@
         <v>84</v>
       </c>
       <c r="K21" s="5"/>
-      <c r="L21" s="4"/>
+      <c r="L21" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="M21" s="5" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="22" spans="2:13" ht="58" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:13" ht="130.5" x14ac:dyDescent="0.35">
       <c r="F22" s="4">
         <v>15</v>
       </c>
@@ -1347,12 +1485,14 @@
         <v>85</v>
       </c>
       <c r="K22" s="5"/>
-      <c r="L22" s="4"/>
+      <c r="L22" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="M22" s="5" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="23" spans="2:13" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:13" ht="159.5" x14ac:dyDescent="0.35">
       <c r="B23" s="1" t="s">
         <v>37</v>
       </c>
@@ -1373,7 +1513,9 @@
       </c>
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
-      <c r="L23" s="4"/>
+      <c r="L23" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="M23" s="5" t="s">
         <v>61</v>
       </c>

</xml_diff>